<commit_message>
tabla y homogenizando nombres
</commit_message>
<xml_diff>
--- a/Numex_preliminar_base.xlsx
+++ b/Numex_preliminar_base.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13725" windowHeight="5235"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6420"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -69,10 +69,10 @@
     <t>height_2024</t>
   </si>
   <si>
-    <t>mean_toughness_(kN/m)</t>
-  </si>
-  <si>
-    <t>mean_thickness_(mm)</t>
+    <t>mean toughness (kN/m)</t>
+  </si>
+  <si>
+    <t>mean thickness (mm)</t>
   </si>
   <si>
     <t>Leaf fresh weight (g)</t>
@@ -84,7 +84,7 @@
     <t>Leaf area (cm²)</t>
   </si>
   <si>
-    <t>SLA (cm²/g)</t>
+    <t>Specific leaf area (g/cm²)</t>
   </si>
   <si>
     <t>area_basal_m2</t>
@@ -96,10 +96,10 @@
     <t>N_P</t>
   </si>
   <si>
-    <t xml:space="preserve">SLA </t>
-  </si>
-  <si>
     <t>code</t>
+  </si>
+  <si>
+    <t>C:N</t>
   </si>
   <si>
     <t>C</t>
@@ -1518,6 +1518,9 @@
       <c r="X2">
         <v>1.276762889372977E-2</v>
       </c>
+      <c r="AB2">
+        <v>39.584547965584058</v>
+      </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
@@ -1592,6 +1595,9 @@
       <c r="X3">
         <v>1.25482750406745E-2</v>
       </c>
+      <c r="AB3">
+        <v>25.578737177957169</v>
+      </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
@@ -1666,6 +1672,9 @@
       <c r="X4">
         <v>8.2676979705257232E-3</v>
       </c>
+      <c r="AB4">
+        <v>42.491614576662137</v>
+      </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1740,6 +1749,9 @@
       <c r="X5">
         <v>0.19011662102463989</v>
       </c>
+      <c r="AB5">
+        <v>29.474945365841709</v>
+      </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
@@ -1814,6 +1826,9 @@
       <c r="X6">
         <v>1.7180121439402771E-2</v>
       </c>
+      <c r="AB6">
+        <v>29.46857519135586</v>
+      </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
@@ -1888,6 +1903,9 @@
       <c r="X7">
         <v>4.4178646691106467E-3</v>
       </c>
+      <c r="AB7">
+        <v>26.51846199848627</v>
+      </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
@@ -1962,6 +1980,9 @@
       <c r="X8">
         <v>3.9478541337997317E-2</v>
       </c>
+      <c r="AB8">
+        <v>29.750151134517079</v>
+      </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -2036,6 +2057,9 @@
       <c r="X9">
         <v>5.9958623116657339E-2</v>
       </c>
+      <c r="AB9">
+        <v>28.284245145374729</v>
+      </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -2110,6 +2134,9 @@
       <c r="X10">
         <v>1.2271846303085129E-2</v>
       </c>
+      <c r="AB10">
+        <v>28.01632724421026</v>
+      </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
@@ -2184,6 +2211,9 @@
       <c r="X11">
         <v>1.414473817944922E-2</v>
       </c>
+      <c r="AB11">
+        <v>39.940382977690383</v>
+      </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -2258,6 +2288,9 @@
       <c r="X12">
         <v>9.7642663168979269E-3</v>
       </c>
+      <c r="AB12">
+        <v>41.333982603305017</v>
+      </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -2332,6 +2365,9 @@
       <c r="X13">
         <v>2.2698006922186251E-2</v>
       </c>
+      <c r="AB13">
+        <v>33.269623957022539</v>
+      </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
@@ -2406,6 +2442,9 @@
       <c r="X14">
         <v>1.9634954084936209E-3</v>
       </c>
+      <c r="AB14">
+        <v>24.516119014230171</v>
+      </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -2480,6 +2519,9 @@
       <c r="X15">
         <v>4.0720766343134887E-2</v>
       </c>
+      <c r="AB15">
+        <v>29.777488603253641</v>
+      </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
@@ -2554,8 +2596,11 @@
       <c r="X16">
         <v>0.1237858191349084</v>
       </c>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB16">
+        <v>32.325474868729572</v>
+      </c>
+    </row>
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -2628,8 +2673,11 @@
       <c r="X17">
         <v>6.8075249750453566E-3</v>
       </c>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB17">
+        <v>28.394486486156119</v>
+      </c>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -2702,8 +2750,11 @@
       <c r="X18">
         <v>7.0685834705770348E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB18">
+        <v>29.176538512475481</v>
+      </c>
+    </row>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -2776,8 +2827,11 @@
       <c r="X19">
         <v>1.504395624468623E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB19">
+        <v>26.667764426662121</v>
+      </c>
+    </row>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -2850,8 +2904,11 @@
       <c r="X20">
         <v>4.6148236789348047E-2</v>
       </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB20">
+        <v>30.754362751178139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -2924,8 +2981,11 @@
       <c r="X21">
         <v>7.9643222219501902E-3</v>
       </c>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB21">
+        <v>22.954085965749901</v>
+      </c>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -2998,8 +3058,11 @@
       <c r="X22">
         <v>2.5929833970768791E-2</v>
       </c>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB22">
+        <v>53.025788268818729</v>
+      </c>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -3072,8 +3135,11 @@
       <c r="X23">
         <v>2.208798031469382E-2</v>
       </c>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB23">
+        <v>38.383701769443327</v>
+      </c>
+    </row>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -3146,8 +3212,11 @@
       <c r="X24">
         <v>4.0715040790523724E-3</v>
       </c>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB24">
+        <v>30.952584320835509</v>
+      </c>
+    </row>
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -3220,8 +3289,11 @@
       <c r="X25">
         <v>0.1164156427695868</v>
       </c>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB25">
+        <v>30.76750734875213</v>
+      </c>
+    </row>
+    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -3294,8 +3366,11 @@
       <c r="X26">
         <v>3.5733173846295721E-2</v>
       </c>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB26">
+        <v>29.191608700076969</v>
+      </c>
+    </row>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -3368,8 +3443,11 @@
       <c r="X27">
         <v>7.9422603875403563E-2</v>
       </c>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB27">
+        <v>19.367486699691309</v>
+      </c>
+    </row>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -3442,8 +3520,11 @@
       <c r="X28">
         <v>4.0715040790523724E-3</v>
       </c>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB28">
+        <v>31.825007955266589</v>
+      </c>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -3516,8 +3597,11 @@
       <c r="X29">
         <v>1.07145902406272E-2</v>
       </c>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB29">
+        <v>20.742167067636121</v>
+      </c>
+    </row>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -3590,8 +3674,11 @@
       <c r="X30">
         <v>2.904346644974163E-2</v>
       </c>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB30">
+        <v>29.191893197903351</v>
+      </c>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -3664,8 +3751,11 @@
       <c r="X31">
         <v>8.5439460665375066E-3</v>
       </c>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB31">
+        <v>42.97256368979243</v>
+      </c>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -3738,8 +3828,11 @@
       <c r="X32">
         <v>5.603219778634775E-2</v>
       </c>
-    </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB32">
+        <v>20.620226785425981</v>
+      </c>
+    </row>
+    <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -3812,8 +3905,11 @@
       <c r="X33">
         <v>0.1092716610753235</v>
       </c>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB33">
+        <v>21.991154966366061</v>
+      </c>
+    </row>
+    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -3886,8 +3982,11 @@
       <c r="X34">
         <v>5.6747719075147723E-2</v>
       </c>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB34">
+        <v>43.871859254690051</v>
+      </c>
+    </row>
+    <row r="35" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -3960,8 +4059,11 @@
       <c r="X35">
         <v>1.278766440087804E-2</v>
       </c>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB35">
+        <v>24.17983322666046</v>
+      </c>
+    </row>
+    <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -4034,8 +4136,11 @@
       <c r="X36">
         <v>9.7642663168979269E-3</v>
       </c>
-    </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB36">
+        <v>45.721716016385123</v>
+      </c>
+    </row>
+    <row r="37" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -4108,8 +4213,11 @@
       <c r="X37">
         <v>1.115943976037552E-2</v>
       </c>
-    </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB37">
+        <v>32.47607689365352</v>
+      </c>
+    </row>
+    <row r="38" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -4182,8 +4290,11 @@
       <c r="X38">
         <v>2.042820622996763E-3</v>
       </c>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB38">
+        <v>31.24223026798138</v>
+      </c>
+    </row>
+    <row r="39" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -4256,8 +4367,11 @@
       <c r="X39">
         <v>7.3013762716062011E-2</v>
       </c>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB39">
+        <v>22.290744965440979</v>
+      </c>
+    </row>
+    <row r="40" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -4330,8 +4444,11 @@
       <c r="X40">
         <v>1.615058225691323E-2</v>
       </c>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB40">
+        <v>40.957146022503892</v>
+      </c>
+    </row>
+    <row r="41" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -4404,8 +4521,11 @@
       <c r="X41">
         <v>1.4762665892465429E-2</v>
       </c>
-    </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB41">
+        <v>32.650535129490073</v>
+      </c>
+    </row>
+    <row r="42" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -4478,8 +4598,11 @@
       <c r="X42">
         <v>1.4762665892465429E-2</v>
       </c>
-    </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB42">
+        <v>32.650535129490073</v>
+      </c>
+    </row>
+    <row r="43" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -4552,8 +4675,11 @@
       <c r="X43">
         <v>1.4762665892465429E-2</v>
       </c>
-    </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB43">
+        <v>32.650535129490073</v>
+      </c>
+    </row>
+    <row r="44" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -4626,8 +4752,11 @@
       <c r="X44">
         <v>1.4762665892465429E-2</v>
       </c>
-    </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB44">
+        <v>32.650535129490073</v>
+      </c>
+    </row>
+    <row r="45" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -4700,8 +4829,11 @@
       <c r="X45">
         <v>8.4459283757455043E-3</v>
       </c>
-    </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB45">
+        <v>34.948373535048873</v>
+      </c>
+    </row>
+    <row r="46" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -4774,8 +4906,11 @@
       <c r="X46">
         <v>1.66728170577011E-2</v>
       </c>
-    </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB46">
+        <v>27.619401676462939</v>
+      </c>
+    </row>
+    <row r="47" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -4848,8 +4983,11 @@
       <c r="X47">
         <v>3.9057065267591708E-2</v>
       </c>
-    </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB47">
+        <v>31.611140549732589</v>
+      </c>
+    </row>
+    <row r="48" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -4922,8 +5060,11 @@
       <c r="X48">
         <v>9.2118486646906965E-3</v>
       </c>
-    </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB48">
+        <v>32.582592220166482</v>
+      </c>
+    </row>
+    <row r="49" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -4996,8 +5137,11 @@
       <c r="X49">
         <v>3.4012146558806168E-2</v>
       </c>
-    </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB49">
+        <v>37.101695936591312</v>
+      </c>
+    </row>
+    <row r="50" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -5070,8 +5214,11 @@
       <c r="X50">
         <v>1.437756946498839E-2</v>
       </c>
-    </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB50">
+        <v>46.620613184773667</v>
+      </c>
+    </row>
+    <row r="51" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -5144,8 +5291,11 @@
       <c r="X51">
         <v>3.4211943997592841E-3</v>
       </c>
-    </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB51">
+        <v>27.642527453599389</v>
+      </c>
+    </row>
+    <row r="52" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -5218,8 +5368,11 @@
       <c r="X52">
         <v>2.7339710067865171E-3</v>
       </c>
-    </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB52">
+        <v>31.43663314688067</v>
+      </c>
+    </row>
+    <row r="53" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -5292,8 +5445,11 @@
       <c r="X53">
         <v>9.7642663168979269E-3</v>
       </c>
-    </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB53">
+        <v>16.47515809594595</v>
+      </c>
+    </row>
+    <row r="54" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -5366,8 +5522,11 @@
       <c r="X54">
         <v>6.7702075667096906E-2</v>
       </c>
-    </row>
-    <row r="55" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB54">
+        <v>17.18961723916043</v>
+      </c>
+    </row>
+    <row r="55" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>53</v>
       </c>
@@ -5440,8 +5599,11 @@
       <c r="X55">
         <v>1.7349445429449631E-3</v>
       </c>
-    </row>
-    <row r="56" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB55">
+        <v>34.169163199183309</v>
+      </c>
+    </row>
+    <row r="56" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>54</v>
       </c>
@@ -5514,8 +5676,11 @@
       <c r="X56">
         <v>1.435632444466849E-2</v>
       </c>
-    </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB56">
+        <v>31.13148059335148</v>
+      </c>
+    </row>
+    <row r="57" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>55</v>
       </c>
@@ -5588,8 +5753,11 @@
       <c r="X57">
         <v>9.3999279628794816E-3</v>
       </c>
-    </row>
-    <row r="58" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB57">
+        <v>42.282611694305608</v>
+      </c>
+    </row>
+    <row r="58" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>56</v>
       </c>
@@ -5662,8 +5830,11 @@
       <c r="X58">
         <v>2.1538256578187049E-2</v>
       </c>
-    </row>
-    <row r="59" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB58">
+        <v>30.408373540103501</v>
+      </c>
+    </row>
+    <row r="59" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>57</v>
       </c>
@@ -5736,8 +5907,11 @@
       <c r="X59">
         <v>1.3872024375172719E-2</v>
       </c>
-    </row>
-    <row r="60" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB59">
+        <v>41.393884528251277</v>
+      </c>
+    </row>
+    <row r="60" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>58</v>
       </c>
@@ -5810,8 +5984,11 @@
       <c r="X60">
         <v>2.1237166338267002E-3</v>
       </c>
-    </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB60">
+        <v>28.161069556696852</v>
+      </c>
+    </row>
+    <row r="61" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>59</v>
       </c>
@@ -5884,8 +6061,11 @@
       <c r="X61">
         <v>3.685284532201676E-3</v>
       </c>
-    </row>
-    <row r="62" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB61">
+        <v>28.349641444429668</v>
+      </c>
+    </row>
+    <row r="62" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>60</v>
       </c>
@@ -5958,8 +6138,11 @@
       <c r="X62">
         <v>0.34315695094977638</v>
       </c>
-    </row>
-    <row r="63" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB62">
+        <v>35.750550975415003</v>
+      </c>
+    </row>
+    <row r="63" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>61</v>
       </c>
@@ -6032,8 +6215,11 @@
       <c r="X63">
         <v>1.5836768566746151E-2</v>
       </c>
-    </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB63">
+        <v>31.74524498440573</v>
+      </c>
+    </row>
+    <row r="64" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>62</v>
       </c>
@@ -6100,8 +6286,11 @@
       <c r="X64">
         <v>1.5836768566746151E-2</v>
       </c>
-    </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB64">
+        <v>32.754821575180422</v>
+      </c>
+    </row>
+    <row r="65" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>63</v>
       </c>
@@ -6174,8 +6363,11 @@
       <c r="X65">
         <v>8.90818231879471E-3</v>
       </c>
-    </row>
-    <row r="66" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB65">
+        <v>37.779784432387643</v>
+      </c>
+    </row>
+    <row r="66" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>64</v>
       </c>
@@ -6248,8 +6440,11 @@
       <c r="X66">
         <v>1.399756241761017E-2</v>
       </c>
-    </row>
-    <row r="67" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB66">
+        <v>46.789905187999963</v>
+      </c>
+    </row>
+    <row r="67" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>65</v>
       </c>
@@ -6322,8 +6517,11 @@
       <c r="X67">
         <v>1.9634954084936209E-3</v>
       </c>
-    </row>
-    <row r="68" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB67">
+        <v>29.55848025895564</v>
+      </c>
+    </row>
+    <row r="68" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>66</v>
       </c>
@@ -6396,8 +6594,11 @@
       <c r="X68">
         <v>2.9224665660019041E-3</v>
       </c>
-    </row>
-    <row r="69" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB68">
+        <v>27.95108301698842</v>
+      </c>
+    </row>
+    <row r="69" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>67</v>
       </c>
@@ -6470,8 +6671,11 @@
       <c r="X69">
         <v>9.8200657148146617E-2</v>
       </c>
-    </row>
-    <row r="70" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB69">
+        <v>24.10341074609785</v>
+      </c>
+    </row>
+    <row r="70" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>68</v>
       </c>
@@ -6544,8 +6748,11 @@
       <c r="X70">
         <v>4.7761287537333733E-2</v>
       </c>
-    </row>
-    <row r="71" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB70">
+        <v>33.078694854662032</v>
+      </c>
+    </row>
+    <row r="71" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>69</v>
       </c>
@@ -6618,8 +6825,11 @@
       <c r="X71">
         <v>2.613000840067389E-2</v>
       </c>
-    </row>
-    <row r="72" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB71">
+        <v>28.437724661298819</v>
+      </c>
+    </row>
+    <row r="72" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>70</v>
       </c>
@@ -6692,8 +6902,11 @@
       <c r="X72">
         <v>2.4744950885540851E-2</v>
       </c>
-    </row>
-    <row r="73" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB72">
+        <v>27.25954615592946</v>
+      </c>
+    </row>
+    <row r="73" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>71</v>
       </c>
@@ -6766,8 +6979,11 @@
       <c r="X73">
         <v>3.1172453105244718E-3</v>
       </c>
-    </row>
-    <row r="74" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB73">
+        <v>30.02082045458015</v>
+      </c>
+    </row>
+    <row r="74" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>72</v>
       </c>
@@ -6840,8 +7056,11 @@
       <c r="X74">
         <v>2.7339710067865171E-3</v>
       </c>
-    </row>
-    <row r="75" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB74">
+        <v>26.467076799846829</v>
+      </c>
+    </row>
+    <row r="75" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>73</v>
       </c>
@@ -6914,8 +7133,11 @@
       <c r="X75">
         <v>0.1121021103925018</v>
       </c>
-    </row>
-    <row r="76" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB75">
+        <v>30.221242016218561</v>
+      </c>
+    </row>
+    <row r="76" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>74</v>
       </c>
@@ -6988,8 +7210,11 @@
       <c r="X76">
         <v>8.5529859993982102E-4</v>
       </c>
-    </row>
-    <row r="77" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB76">
+        <v>32.733361647666023</v>
+      </c>
+    </row>
+    <row r="77" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>75</v>
       </c>
@@ -7062,8 +7287,11 @@
       <c r="X77">
         <v>9.0792027688745003E-4</v>
       </c>
-    </row>
-    <row r="78" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB77">
+        <v>27.859584291279319</v>
+      </c>
+    </row>
+    <row r="78" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>76</v>
       </c>
@@ -7136,8 +7364,11 @@
       <c r="X78">
         <v>2.3289286075518389E-2</v>
       </c>
-    </row>
-    <row r="79" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB78">
+        <v>21.816209618740601</v>
+      </c>
+    </row>
+    <row r="79" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>77</v>
       </c>
@@ -7210,8 +7441,11 @@
       <c r="X79">
         <v>1.020703453151324E-2</v>
       </c>
-    </row>
-    <row r="80" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="AB79">
+        <v>18.284786480705879</v>
+      </c>
+    </row>
+    <row r="80" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>78</v>
       </c>
@@ -7283,6 +7517,9 @@
       </c>
       <c r="X80">
         <v>3.6170067282648828E-2</v>
+      </c>
+      <c r="AB80">
+        <v>22.129089554863011</v>
       </c>
     </row>
     <row r="81" spans="1:28" x14ac:dyDescent="0.25">
@@ -7358,6 +7595,9 @@
       <c r="X81">
         <v>5.6200147329608659E-2</v>
       </c>
+      <c r="AB81">
+        <v>23.887729422282892</v>
+      </c>
     </row>
     <row r="82" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
@@ -7432,6 +7672,9 @@
       <c r="X82">
         <v>1.459088360616714E-2</v>
       </c>
+      <c r="AB82">
+        <v>29.221428889168031</v>
+      </c>
     </row>
     <row r="83" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
@@ -7506,6 +7749,9 @@
       <c r="X83">
         <v>8.0436081665451603E-3</v>
       </c>
+      <c r="AB83">
+        <v>26.316250120372359</v>
+      </c>
     </row>
     <row r="84" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
@@ -7580,6 +7826,9 @@
       <c r="X84">
         <v>8.4133814758543136E-3</v>
       </c>
+      <c r="AB84">
+        <v>30.204164678379829</v>
+      </c>
     </row>
     <row r="85" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
@@ -7654,6 +7903,9 @@
       <c r="X85">
         <v>7.6551847924479735E-2</v>
       </c>
+      <c r="AB85">
+        <v>27.98331631734705</v>
+      </c>
     </row>
     <row r="86" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
@@ -7728,6 +7980,9 @@
       <c r="X86">
         <v>8.4341780338229186E-2</v>
       </c>
+      <c r="AB86">
+        <v>30.59860950966031</v>
+      </c>
     </row>
     <row r="87" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
@@ -7802,6 +8057,9 @@
       <c r="X87">
         <v>2.7339710067865171E-3</v>
       </c>
+      <c r="AB87">
+        <v>27.00689943428555</v>
+      </c>
     </row>
     <row r="88" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
@@ -7876,6 +8134,9 @@
       <c r="X88">
         <v>4.1692201769496277E-2</v>
       </c>
+      <c r="AB88">
+        <v>20.099816088682122</v>
+      </c>
     </row>
     <row r="89" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
@@ -7932,8 +8193,11 @@
       <c r="S89">
         <v>0.48099999999999998</v>
       </c>
-      <c r="AB89" t="s">
+      <c r="AA89" t="s">
         <v>125</v>
+      </c>
+      <c r="AB89">
+        <v>59.387164735194609</v>
       </c>
     </row>
     <row r="90" spans="1:28" x14ac:dyDescent="0.25">
@@ -7991,8 +8255,11 @@
       <c r="S90">
         <v>0.42983333333333329</v>
       </c>
-      <c r="AB90" t="s">
+      <c r="AA90" t="s">
         <v>128</v>
+      </c>
+      <c r="AB90">
+        <v>55.075494177356553</v>
       </c>
     </row>
     <row r="91" spans="1:28" x14ac:dyDescent="0.25">
@@ -8050,8 +8317,11 @@
       <c r="S91">
         <v>0.5006666666666667</v>
       </c>
-      <c r="AB91" t="s">
+      <c r="AA91" t="s">
         <v>130</v>
+      </c>
+      <c r="AB91">
+        <v>45.177578357683032</v>
       </c>
     </row>
     <row r="92" spans="1:28" x14ac:dyDescent="0.25">
@@ -8109,8 +8379,11 @@
       <c r="S92">
         <v>0.53600000000000003</v>
       </c>
-      <c r="AB92" t="s">
+      <c r="AA92" t="s">
         <v>133</v>
+      </c>
+      <c r="AB92">
+        <v>43.386374346901121</v>
       </c>
     </row>
     <row r="93" spans="1:28" x14ac:dyDescent="0.25">
@@ -8168,8 +8441,11 @@
       <c r="S93">
         <v>0.45316666666666672</v>
       </c>
-      <c r="AB93" t="s">
+      <c r="AA93" t="s">
         <v>136</v>
+      </c>
+      <c r="AB93">
+        <v>61.02294354014969</v>
       </c>
     </row>
     <row r="94" spans="1:28" x14ac:dyDescent="0.25">
@@ -8227,8 +8503,11 @@
       <c r="S94">
         <v>0.47449999999999992</v>
       </c>
-      <c r="AB94" t="s">
+      <c r="AA94" t="s">
         <v>139</v>
+      </c>
+      <c r="AB94">
+        <v>50.188888491816037</v>
       </c>
     </row>
     <row r="95" spans="1:28" x14ac:dyDescent="0.25">
@@ -8286,8 +8565,11 @@
       <c r="S95">
         <v>0.626</v>
       </c>
-      <c r="AB95" t="s">
+      <c r="AA95" t="s">
         <v>145</v>
+      </c>
+      <c r="AB95">
+        <v>44.535373568956267</v>
       </c>
     </row>
     <row r="96" spans="1:28" x14ac:dyDescent="0.25">
@@ -8345,8 +8627,11 @@
       <c r="S96">
         <v>0.4335</v>
       </c>
-      <c r="AB96" t="s">
+      <c r="AA96" t="s">
         <v>148</v>
+      </c>
+      <c r="AB96">
+        <v>41.912014933516289</v>
       </c>
     </row>
     <row r="97" spans="1:28" x14ac:dyDescent="0.25">
@@ -8404,8 +8689,11 @@
       <c r="S97">
         <v>0.46633333333333332</v>
       </c>
-      <c r="AB97" t="s">
+      <c r="AA97" t="s">
         <v>151</v>
+      </c>
+      <c r="AB97">
+        <v>70.706126134262732</v>
       </c>
     </row>
     <row r="98" spans="1:28" x14ac:dyDescent="0.25">
@@ -8463,8 +8751,11 @@
       <c r="S98">
         <v>0.45816666666666661</v>
       </c>
-      <c r="AB98" t="s">
+      <c r="AA98" t="s">
         <v>153</v>
+      </c>
+      <c r="AB98">
+        <v>56.157007987138407</v>
       </c>
     </row>
     <row r="99" spans="1:28" x14ac:dyDescent="0.25">
@@ -8522,8 +8813,11 @@
       <c r="S99">
         <v>0.40433333333333332</v>
       </c>
-      <c r="AB99" t="s">
+      <c r="AA99" t="s">
         <v>155</v>
+      </c>
+      <c r="AB99">
+        <v>55.792464496669943</v>
       </c>
     </row>
     <row r="100" spans="1:28" x14ac:dyDescent="0.25">
@@ -8581,8 +8875,11 @@
       <c r="S100">
         <v>0.4948333333333334</v>
       </c>
-      <c r="AB100" t="s">
+      <c r="AA100" t="s">
         <v>157</v>
+      </c>
+      <c r="AB100">
+        <v>65.934750176804783</v>
       </c>
     </row>
     <row r="101" spans="1:28" x14ac:dyDescent="0.25">
@@ -8640,8 +8937,11 @@
       <c r="S101">
         <v>0.56883333333333341</v>
       </c>
-      <c r="AB101" t="s">
+      <c r="AA101" t="s">
         <v>159</v>
+      </c>
+      <c r="AB101">
+        <v>35.493764344055123</v>
       </c>
     </row>
     <row r="102" spans="1:28" x14ac:dyDescent="0.25">
@@ -8699,8 +8999,11 @@
       <c r="S102">
         <v>0.58350000000000002</v>
       </c>
-      <c r="AB102" t="s">
+      <c r="AA102" t="s">
         <v>161</v>
+      </c>
+      <c r="AB102">
+        <v>62.556868487705593</v>
       </c>
     </row>
     <row r="103" spans="1:28" x14ac:dyDescent="0.25">
@@ -8758,8 +9061,11 @@
       <c r="S103">
         <v>0.46650000000000003</v>
       </c>
-      <c r="AB103" t="s">
+      <c r="AA103" t="s">
         <v>164</v>
+      </c>
+      <c r="AB103">
+        <v>48.184839932225927</v>
       </c>
     </row>
     <row r="104" spans="1:28" x14ac:dyDescent="0.25">
@@ -8817,8 +9123,11 @@
       <c r="S104">
         <v>0.49366666666666659</v>
       </c>
-      <c r="AB104" t="s">
+      <c r="AA104" t="s">
         <v>167</v>
+      </c>
+      <c r="AB104">
+        <v>48.500365054530441</v>
       </c>
     </row>
     <row r="105" spans="1:28" x14ac:dyDescent="0.25">
@@ -8876,8 +9185,11 @@
       <c r="S105">
         <v>0.48316666666666669</v>
       </c>
-      <c r="AB105" t="s">
+      <c r="AA105" t="s">
         <v>170</v>
+      </c>
+      <c r="AB105">
+        <v>48.824057143664227</v>
       </c>
     </row>
     <row r="106" spans="1:28" x14ac:dyDescent="0.25">
@@ -8935,8 +9247,11 @@
       <c r="S106">
         <v>0.46500000000000002</v>
       </c>
-      <c r="AB106" t="s">
+      <c r="AA106" t="s">
         <v>172</v>
+      </c>
+      <c r="AB106">
+        <v>42.085669628700977</v>
       </c>
     </row>
     <row r="107" spans="1:28" x14ac:dyDescent="0.25">
@@ -8994,8 +9309,11 @@
       <c r="S107">
         <v>0.46633333333333332</v>
       </c>
-      <c r="AB107" t="s">
+      <c r="AA107" t="s">
         <v>175</v>
+      </c>
+      <c r="AB107">
+        <v>51.945262955906408</v>
       </c>
     </row>
     <row r="108" spans="1:28" x14ac:dyDescent="0.25">
@@ -9053,8 +9371,11 @@
       <c r="S108">
         <v>0.47233333333333333</v>
       </c>
-      <c r="AB108" t="s">
+      <c r="AA108" t="s">
         <v>178</v>
+      </c>
+      <c r="AB108">
+        <v>55.623935343866329</v>
       </c>
     </row>
     <row r="109" spans="1:28" x14ac:dyDescent="0.25">
@@ -9112,8 +9433,11 @@
       <c r="S109">
         <v>0.48733333333333329</v>
       </c>
-      <c r="AB109" t="s">
+      <c r="AA109" t="s">
         <v>180</v>
+      </c>
+      <c r="AB109">
+        <v>58.951576669977257</v>
       </c>
     </row>
     <row r="110" spans="1:28" x14ac:dyDescent="0.25">
@@ -9171,8 +9495,11 @@
       <c r="S110">
         <v>0.46233333333333332</v>
       </c>
-      <c r="AB110" t="s">
+      <c r="AA110" t="s">
         <v>182</v>
+      </c>
+      <c r="AB110">
+        <v>61.689918975438367</v>
       </c>
     </row>
     <row r="111" spans="1:28" x14ac:dyDescent="0.25">
@@ -9230,8 +9557,11 @@
       <c r="S111">
         <v>0.47983333333333328</v>
       </c>
-      <c r="AB111" t="s">
+      <c r="AA111" t="s">
         <v>184</v>
+      </c>
+      <c r="AB111">
+        <v>42.51564615776595</v>
       </c>
     </row>
     <row r="112" spans="1:28" x14ac:dyDescent="0.25">
@@ -9289,8 +9619,11 @@
       <c r="S112">
         <v>0.53733333333333333</v>
       </c>
-      <c r="AB112" t="s">
+      <c r="AA112" t="s">
         <v>186</v>
+      </c>
+      <c r="AB112">
+        <v>43.639776917431128</v>
       </c>
     </row>
     <row r="113" spans="1:28" x14ac:dyDescent="0.25">
@@ -9348,8 +9681,11 @@
       <c r="S113">
         <v>0.39516666666666672</v>
       </c>
-      <c r="AB113" t="s">
+      <c r="AA113" t="s">
         <v>188</v>
+      </c>
+      <c r="AB113">
+        <v>48.271073415871413</v>
       </c>
     </row>
     <row r="114" spans="1:28" x14ac:dyDescent="0.25">
@@ -9407,8 +9743,11 @@
       <c r="S114">
         <v>0.46500000000000002</v>
       </c>
-      <c r="AB114" t="s">
+      <c r="AA114" t="s">
         <v>190</v>
+      </c>
+      <c r="AB114">
+        <v>55.685332531514931</v>
       </c>
     </row>
     <row r="115" spans="1:28" x14ac:dyDescent="0.25">
@@ -9466,8 +9805,11 @@
       <c r="S115">
         <v>0.49199999999999999</v>
       </c>
-      <c r="AB115" t="s">
+      <c r="AA115" t="s">
         <v>192</v>
+      </c>
+      <c r="AB115">
+        <v>46.552859383739893</v>
       </c>
     </row>
     <row r="116" spans="1:28" x14ac:dyDescent="0.25">
@@ -9525,8 +9867,11 @@
       <c r="S116">
         <v>0.53599999999999992</v>
       </c>
-      <c r="AB116" t="s">
+      <c r="AA116" t="s">
         <v>194</v>
+      </c>
+      <c r="AB116">
+        <v>28.782853440115371</v>
       </c>
     </row>
     <row r="117" spans="1:28" x14ac:dyDescent="0.25">
@@ -9584,8 +9929,11 @@
       <c r="S117">
         <v>0.44216666666666671</v>
       </c>
-      <c r="AB117" t="s">
+      <c r="AA117" t="s">
         <v>196</v>
+      </c>
+      <c r="AB117">
+        <v>40.260960035570477</v>
       </c>
     </row>
     <row r="118" spans="1:28" x14ac:dyDescent="0.25">
@@ -9643,8 +9991,11 @@
       <c r="S118">
         <v>0.44216666666666671</v>
       </c>
-      <c r="AB118" t="s">
+      <c r="AA118" t="s">
         <v>196</v>
+      </c>
+      <c r="AB118">
+        <v>40.260960035570477</v>
       </c>
     </row>
     <row r="119" spans="1:28" x14ac:dyDescent="0.25">
@@ -9702,8 +10053,11 @@
       <c r="S119">
         <v>0.51633333333333331</v>
       </c>
-      <c r="AB119" t="s">
+      <c r="AA119" t="s">
         <v>198</v>
+      </c>
+      <c r="AB119">
+        <v>38.628305463248843</v>
       </c>
     </row>
     <row r="120" spans="1:28" x14ac:dyDescent="0.25">
@@ -9761,8 +10115,11 @@
       <c r="S120">
         <v>0.63350000000000006</v>
       </c>
-      <c r="AB120" t="s">
+      <c r="AA120" t="s">
         <v>200</v>
+      </c>
+      <c r="AB120">
+        <v>47.604435545316143</v>
       </c>
     </row>
     <row r="121" spans="1:28" x14ac:dyDescent="0.25">
@@ -9820,8 +10177,11 @@
       <c r="S121">
         <v>0.63350000000000006</v>
       </c>
-      <c r="AB121" t="s">
+      <c r="AA121" t="s">
         <v>200</v>
+      </c>
+      <c r="AB121">
+        <v>47.604435545316143</v>
       </c>
     </row>
     <row r="122" spans="1:28" x14ac:dyDescent="0.25">
@@ -9879,8 +10239,11 @@
       <c r="S122">
         <v>0.54666666666666675</v>
       </c>
-      <c r="AB122" t="s">
+      <c r="AA122" t="s">
         <v>202</v>
+      </c>
+      <c r="AB122">
+        <v>38.09610849251812</v>
       </c>
     </row>
     <row r="123" spans="1:28" x14ac:dyDescent="0.25">
@@ -9938,8 +10301,11 @@
       <c r="S123">
         <v>0.52133333333333332</v>
       </c>
-      <c r="AB123" t="s">
+      <c r="AA123" t="s">
         <v>204</v>
+      </c>
+      <c r="AB123">
+        <v>35.84967061566433</v>
       </c>
     </row>
     <row r="124" spans="1:28" x14ac:dyDescent="0.25">
@@ -9997,8 +10363,11 @@
       <c r="S124">
         <v>0.57550000000000001</v>
       </c>
-      <c r="AB124" t="s">
+      <c r="AA124" t="s">
         <v>206</v>
+      </c>
+      <c r="AB124">
+        <v>46.885815862684261</v>
       </c>
     </row>
     <row r="125" spans="1:28" x14ac:dyDescent="0.25">
@@ -10056,8 +10425,11 @@
       <c r="S125">
         <v>0.57366666666666666</v>
       </c>
-      <c r="AB125" t="s">
+      <c r="AA125" t="s">
         <v>208</v>
+      </c>
+      <c r="AB125">
+        <v>51.208086139015798</v>
       </c>
     </row>
     <row r="126" spans="1:28" x14ac:dyDescent="0.25">
@@ -10115,8 +10487,11 @@
       <c r="S126">
         <v>0.46516666666666667</v>
       </c>
-      <c r="AB126" t="s">
+      <c r="AA126" t="s">
         <v>211</v>
+      </c>
+      <c r="AB126">
+        <v>44.756239097433053</v>
       </c>
     </row>
     <row r="127" spans="1:28" x14ac:dyDescent="0.25">
@@ -10174,8 +10549,11 @@
       <c r="S127">
         <v>0.50383333333333324</v>
       </c>
-      <c r="AB127" t="s">
+      <c r="AA127" t="s">
         <v>213</v>
+      </c>
+      <c r="AB127">
+        <v>38.485721162919504</v>
       </c>
     </row>
     <row r="128" spans="1:28" x14ac:dyDescent="0.25">
@@ -10233,8 +10611,11 @@
       <c r="S128">
         <v>0.5635</v>
       </c>
-      <c r="AB128" t="s">
+      <c r="AA128" t="s">
         <v>215</v>
+      </c>
+      <c r="AB128">
+        <v>38.028812877437822</v>
       </c>
     </row>
     <row r="129" spans="1:28" x14ac:dyDescent="0.25">
@@ -10292,8 +10673,11 @@
       <c r="S129">
         <v>0.57916666666666672</v>
       </c>
-      <c r="AB129" t="s">
+      <c r="AA129" t="s">
         <v>217</v>
+      </c>
+      <c r="AB129">
+        <v>42.691616333196791</v>
       </c>
     </row>
     <row r="130" spans="1:28" x14ac:dyDescent="0.25">
@@ -10351,8 +10735,11 @@
       <c r="S130">
         <v>0.59083333333333332</v>
       </c>
-      <c r="AB130" t="s">
+      <c r="AA130" t="s">
         <v>219</v>
+      </c>
+      <c r="AB130">
+        <v>42.92451945516472</v>
       </c>
     </row>
     <row r="131" spans="1:28" x14ac:dyDescent="0.25">
@@ -10410,8 +10797,11 @@
       <c r="S131">
         <v>0.53949999999999998</v>
       </c>
-      <c r="AB131" t="s">
+      <c r="AA131" t="s">
         <v>222</v>
+      </c>
+      <c r="AB131">
+        <v>40.164799058724142</v>
       </c>
     </row>
     <row r="132" spans="1:28" x14ac:dyDescent="0.25">
@@ -10469,8 +10859,11 @@
       <c r="S132">
         <v>0.4955</v>
       </c>
-      <c r="AB132" t="s">
+      <c r="AA132" t="s">
         <v>224</v>
+      </c>
+      <c r="AB132">
+        <v>54.145542178910453</v>
       </c>
     </row>
     <row r="133" spans="1:28" x14ac:dyDescent="0.25">
@@ -10528,8 +10921,11 @@
       <c r="S133">
         <v>0.4955</v>
       </c>
-      <c r="AB133" t="s">
+      <c r="AA133" t="s">
         <v>224</v>
+      </c>
+      <c r="AB133">
+        <v>54.145542178910453</v>
       </c>
     </row>
     <row r="134" spans="1:28" x14ac:dyDescent="0.25">
@@ -10587,8 +10983,11 @@
       <c r="S134">
         <v>0.53433333333333333</v>
       </c>
-      <c r="AB134" t="s">
+      <c r="AA134" t="s">
         <v>226</v>
+      </c>
+      <c r="AB134">
+        <v>34.630306316877338</v>
       </c>
     </row>
     <row r="135" spans="1:28" x14ac:dyDescent="0.25">
@@ -10646,8 +11045,11 @@
       <c r="S135">
         <v>0.56933333333333336</v>
       </c>
-      <c r="AB135" t="s">
+      <c r="AA135" t="s">
         <v>228</v>
+      </c>
+      <c r="AB135">
+        <v>44.899969358384858</v>
       </c>
     </row>
     <row r="136" spans="1:28" x14ac:dyDescent="0.25">
@@ -10705,8 +11107,11 @@
       <c r="S136">
         <v>0.5053333333333333</v>
       </c>
-      <c r="AB136" t="s">
+      <c r="AA136" t="s">
         <v>230</v>
+      </c>
+      <c r="AB136">
+        <v>43.934199060950966</v>
       </c>
     </row>
     <row r="137" spans="1:28" x14ac:dyDescent="0.25">
@@ -10764,8 +11169,11 @@
       <c r="S137">
         <v>0.42333333333333328</v>
       </c>
-      <c r="AB137" t="s">
+      <c r="AA137" t="s">
         <v>232</v>
+      </c>
+      <c r="AB137">
+        <v>62.739747321720387</v>
       </c>
     </row>
     <row r="138" spans="1:28" x14ac:dyDescent="0.25">
@@ -10823,8 +11231,11 @@
       <c r="S138">
         <v>0.51316666666666666</v>
       </c>
-      <c r="AB138" t="s">
+      <c r="AA138" t="s">
         <v>234</v>
+      </c>
+      <c r="AB138">
+        <v>56.825935297343378</v>
       </c>
     </row>
     <row r="139" spans="1:28" x14ac:dyDescent="0.25">
@@ -10882,8 +11293,11 @@
       <c r="S139">
         <v>0.4988333333333333</v>
       </c>
-      <c r="AB139" t="s">
+      <c r="AA139" t="s">
         <v>236</v>
+      </c>
+      <c r="AB139">
+        <v>51.971564573205853</v>
       </c>
     </row>
     <row r="140" spans="1:28" x14ac:dyDescent="0.25">
@@ -10941,8 +11355,11 @@
       <c r="S140">
         <v>0.48566666666666658</v>
       </c>
-      <c r="AB140" t="s">
+      <c r="AA140" t="s">
         <v>239</v>
+      </c>
+      <c r="AB140">
+        <v>34.71279366258031</v>
       </c>
     </row>
     <row r="141" spans="1:28" x14ac:dyDescent="0.25">
@@ -11000,8 +11417,11 @@
       <c r="S141">
         <v>0.46516666666666667</v>
       </c>
-      <c r="AB141" t="s">
+      <c r="AA141" t="s">
         <v>241</v>
+      </c>
+      <c r="AB141">
+        <v>16.82978356315537</v>
       </c>
     </row>
     <row r="142" spans="1:28" x14ac:dyDescent="0.25">
@@ -11059,8 +11479,11 @@
       <c r="S142">
         <v>0.47949999999999998</v>
       </c>
-      <c r="AB142" t="s">
+      <c r="AA142" t="s">
         <v>243</v>
+      </c>
+      <c r="AB142">
+        <v>48.866625295567033</v>
       </c>
     </row>
     <row r="143" spans="1:28" x14ac:dyDescent="0.25">
@@ -11118,8 +11541,11 @@
       <c r="S143">
         <v>0.48549999999999999</v>
       </c>
-      <c r="AB143" t="s">
+      <c r="AA143" t="s">
         <v>245</v>
+      </c>
+      <c r="AB143">
+        <v>48.489895803794177</v>
       </c>
     </row>
     <row r="144" spans="1:28" x14ac:dyDescent="0.25">
@@ -11177,8 +11603,11 @@
       <c r="S144">
         <v>0.49299999999999988</v>
       </c>
-      <c r="AB144" t="s">
+      <c r="AA144" t="s">
         <v>247</v>
+      </c>
+      <c r="AB144">
+        <v>52.455135383105983</v>
       </c>
     </row>
     <row r="145" spans="1:28" x14ac:dyDescent="0.25">
@@ -11236,8 +11665,11 @@
       <c r="S145">
         <v>0.47383333333333327</v>
       </c>
-      <c r="AB145" t="s">
+      <c r="AA145" t="s">
         <v>249</v>
+      </c>
+      <c r="AB145">
+        <v>50.12173210626537</v>
       </c>
     </row>
     <row r="146" spans="1:28" x14ac:dyDescent="0.25">
@@ -11295,8 +11727,11 @@
       <c r="S146">
         <v>0.48699999999999988</v>
       </c>
-      <c r="AB146" t="s">
+      <c r="AA146" t="s">
         <v>251</v>
+      </c>
+      <c r="AB146">
+        <v>51.649055858324083</v>
       </c>
     </row>
     <row r="147" spans="1:28" x14ac:dyDescent="0.25">
@@ -11354,8 +11789,11 @@
       <c r="S147">
         <v>0.42983333333333329</v>
       </c>
-      <c r="AB147" t="s">
+      <c r="AA147" t="s">
         <v>253</v>
+      </c>
+      <c r="AB147">
+        <v>40.845732336609991</v>
       </c>
     </row>
     <row r="148" spans="1:28" x14ac:dyDescent="0.25">
@@ -11413,8 +11851,11 @@
       <c r="S148">
         <v>0.5528333333333334</v>
       </c>
-      <c r="AB148" t="s">
+      <c r="AA148" t="s">
         <v>255</v>
+      </c>
+      <c r="AB148">
+        <v>37.419618751843892</v>
       </c>
     </row>
     <row r="149" spans="1:28" x14ac:dyDescent="0.25">
@@ -11472,8 +11913,11 @@
       <c r="S149">
         <v>0.50579999999999992</v>
       </c>
-      <c r="AB149" t="s">
+      <c r="AA149" t="s">
         <v>257</v>
+      </c>
+      <c r="AB149">
+        <v>44.985940912182429</v>
       </c>
     </row>
     <row r="150" spans="1:28" x14ac:dyDescent="0.25">
@@ -11531,8 +11975,11 @@
       <c r="S150">
         <v>0.4928333333333334</v>
       </c>
-      <c r="AB150" t="s">
+      <c r="AA150" t="s">
         <v>259</v>
+      </c>
+      <c r="AB150">
+        <v>62.328759010480503</v>
       </c>
     </row>
     <row r="151" spans="1:28" x14ac:dyDescent="0.25">
@@ -11590,8 +12037,11 @@
       <c r="S151">
         <v>0.45116666666666672</v>
       </c>
-      <c r="AB151" t="s">
+      <c r="AA151" t="s">
         <v>261</v>
+      </c>
+      <c r="AB151">
+        <v>63.04106431069755</v>
       </c>
     </row>
     <row r="152" spans="1:28" x14ac:dyDescent="0.25">
@@ -11649,8 +12099,11 @@
       <c r="S152">
         <v>0.47699999999999992</v>
       </c>
-      <c r="AB152" t="s">
+      <c r="AA152" t="s">
         <v>263</v>
+      </c>
+      <c r="AB152">
+        <v>55.566677261637743</v>
       </c>
     </row>
     <row r="153" spans="1:28" x14ac:dyDescent="0.25">
@@ -11708,8 +12161,11 @@
       <c r="S153">
         <v>0.48849999999999999</v>
       </c>
-      <c r="AB153" t="s">
+      <c r="AA153" t="s">
         <v>265</v>
+      </c>
+      <c r="AB153">
+        <v>61.707998069625013</v>
       </c>
     </row>
     <row r="154" spans="1:28" x14ac:dyDescent="0.25">
@@ -11767,8 +12223,11 @@
       <c r="S154">
         <v>0.48</v>
       </c>
-      <c r="AB154" t="s">
+      <c r="AA154" t="s">
         <v>267</v>
+      </c>
+      <c r="AB154">
+        <v>47.273238556076549</v>
       </c>
     </row>
     <row r="155" spans="1:28" x14ac:dyDescent="0.25">
@@ -11826,8 +12285,11 @@
       <c r="S155">
         <v>0.45800000000000002</v>
       </c>
-      <c r="AB155" t="s">
+      <c r="AA155" t="s">
         <v>269</v>
+      </c>
+      <c r="AB155">
+        <v>46.600210452192208</v>
       </c>
     </row>
     <row r="156" spans="1:28" x14ac:dyDescent="0.25">
@@ -11885,8 +12347,11 @@
       <c r="S156">
         <v>0.57333333333333325</v>
       </c>
-      <c r="AB156" t="s">
+      <c r="AA156" t="s">
         <v>271</v>
+      </c>
+      <c r="AB156">
+        <v>36.4008599384631</v>
       </c>
     </row>
     <row r="157" spans="1:28" x14ac:dyDescent="0.25">
@@ -11944,8 +12409,11 @@
       <c r="S157">
         <v>0.46266666666666662</v>
       </c>
-      <c r="AB157" t="s">
+      <c r="AA157" t="s">
         <v>273</v>
+      </c>
+      <c r="AB157">
+        <v>55.608195326274043</v>
       </c>
     </row>
     <row r="158" spans="1:28" x14ac:dyDescent="0.25">
@@ -12003,8 +12471,11 @@
       <c r="S158">
         <v>0.5063333333333333</v>
       </c>
-      <c r="AB158" t="s">
+      <c r="AA158" t="s">
         <v>275</v>
+      </c>
+      <c r="AB158">
+        <v>43.121642980196953</v>
       </c>
     </row>
     <row r="159" spans="1:28" x14ac:dyDescent="0.25">
@@ -12062,8 +12533,11 @@
       <c r="S159">
         <v>0.5063333333333333</v>
       </c>
-      <c r="AB159" t="s">
+      <c r="AA159" t="s">
         <v>275</v>
+      </c>
+      <c r="AB159">
+        <v>43.121642980196953</v>
       </c>
     </row>
     <row r="160" spans="1:28" x14ac:dyDescent="0.25">
@@ -12121,8 +12595,11 @@
       <c r="S160">
         <v>0.4965</v>
       </c>
-      <c r="AB160" t="s">
+      <c r="AA160" t="s">
         <v>277</v>
+      </c>
+      <c r="AB160">
+        <v>40.641455533402819</v>
       </c>
     </row>
     <row r="161" spans="1:28" x14ac:dyDescent="0.25">
@@ -12177,8 +12654,11 @@
       <c r="S161">
         <v>0.50116666666666665</v>
       </c>
-      <c r="AB161" t="s">
+      <c r="AA161" t="s">
         <v>279</v>
+      </c>
+      <c r="AB161">
+        <v>39.863887138589867</v>
       </c>
     </row>
     <row r="162" spans="1:28" x14ac:dyDescent="0.25">
@@ -12233,8 +12713,11 @@
       <c r="S162">
         <v>0.44766666666666671</v>
       </c>
-      <c r="AB162" t="s">
+      <c r="AA162" t="s">
         <v>281</v>
+      </c>
+      <c r="AB162">
+        <v>50.489542564850623</v>
       </c>
     </row>
     <row r="163" spans="1:28" x14ac:dyDescent="0.25">
@@ -12292,8 +12775,11 @@
       <c r="S163">
         <v>0.48799999999999999</v>
       </c>
-      <c r="AB163" t="s">
+      <c r="AA163" t="s">
         <v>283</v>
+      </c>
+      <c r="AB163">
+        <v>53.087250316175677</v>
       </c>
     </row>
     <row r="164" spans="1:28" x14ac:dyDescent="0.25">
@@ -12351,8 +12837,11 @@
       <c r="S164">
         <v>0.4971666666666667</v>
       </c>
-      <c r="AB164" t="s">
+      <c r="AA164" t="s">
         <v>285</v>
+      </c>
+      <c r="AB164">
+        <v>45.200141422627198</v>
       </c>
     </row>
     <row r="165" spans="1:28" x14ac:dyDescent="0.25">
@@ -12410,8 +12899,11 @@
       <c r="S165">
         <v>0.48666666666666669</v>
       </c>
-      <c r="AB165" t="s">
+      <c r="AA165" t="s">
         <v>287</v>
+      </c>
+      <c r="AB165">
+        <v>48.166853356437819</v>
       </c>
     </row>
     <row r="166" spans="1:28" x14ac:dyDescent="0.25">
@@ -12469,8 +12961,11 @@
       <c r="S166">
         <v>0.55649999999999999</v>
       </c>
-      <c r="AB166" t="s">
+      <c r="AA166" t="s">
         <v>289</v>
+      </c>
+      <c r="AB166">
+        <v>42.614255405168286</v>
       </c>
     </row>
     <row r="167" spans="1:28" x14ac:dyDescent="0.25">
@@ -12528,8 +13023,11 @@
       <c r="S167">
         <v>0.42499999999999999</v>
       </c>
-      <c r="AB167" t="s">
+      <c r="AA167" t="s">
         <v>291</v>
+      </c>
+      <c r="AB167">
+        <v>42.469932491000257</v>
       </c>
     </row>
     <row r="168" spans="1:28" x14ac:dyDescent="0.25">
@@ -12587,8 +13085,11 @@
       <c r="S168">
         <v>0.50316666666666665</v>
       </c>
-      <c r="AB168" t="s">
+      <c r="AA168" t="s">
         <v>293</v>
+      </c>
+      <c r="AB168">
+        <v>38.407014171063572</v>
       </c>
     </row>
     <row r="169" spans="1:28" x14ac:dyDescent="0.25">
@@ -12646,8 +13147,11 @@
       <c r="S169">
         <v>0.52666666666666673</v>
       </c>
-      <c r="AB169" t="s">
+      <c r="AA169" t="s">
         <v>295</v>
+      </c>
+      <c r="AB169">
+        <v>41.279671375048508</v>
       </c>
     </row>
     <row r="170" spans="1:28" x14ac:dyDescent="0.25">
@@ -12705,8 +13209,11 @@
       <c r="S170">
         <v>0.58466666666666667</v>
       </c>
-      <c r="AB170" t="s">
+      <c r="AA170" t="s">
         <v>297</v>
+      </c>
+      <c r="AB170">
+        <v>40.637487861761699</v>
       </c>
     </row>
     <row r="171" spans="1:28" x14ac:dyDescent="0.25">
@@ -12764,8 +13271,11 @@
       <c r="S171">
         <v>0.52033333333333331</v>
       </c>
-      <c r="AB171" t="s">
+      <c r="AA171" t="s">
         <v>299</v>
+      </c>
+      <c r="AB171">
+        <v>38.086844726005268</v>
       </c>
     </row>
     <row r="172" spans="1:28" x14ac:dyDescent="0.25">
@@ -12823,8 +13333,11 @@
       <c r="S172">
         <v>0.59766666666666668</v>
       </c>
-      <c r="AB172" t="s">
+      <c r="AA172" t="s">
         <v>301</v>
+      </c>
+      <c r="AB172">
+        <v>43.331083566213067</v>
       </c>
     </row>
     <row r="173" spans="1:28" x14ac:dyDescent="0.25">
@@ -12882,8 +13395,11 @@
       <c r="S173">
         <v>0.45033333333333331</v>
       </c>
-      <c r="AB173" t="s">
+      <c r="AA173" t="s">
         <v>303</v>
+      </c>
+      <c r="AB173">
+        <v>45.597827124848862</v>
       </c>
     </row>
     <row r="174" spans="1:28" x14ac:dyDescent="0.25">
@@ -12941,8 +13457,11 @@
       <c r="S174">
         <v>0.47266666666666662</v>
       </c>
-      <c r="AB174" t="s">
+      <c r="AA174" t="s">
         <v>305</v>
+      </c>
+      <c r="AB174">
+        <v>46.088628516364693</v>
       </c>
     </row>
     <row r="175" spans="1:28" x14ac:dyDescent="0.25">
@@ -13000,8 +13519,11 @@
       <c r="S175">
         <v>0.54099999999999993</v>
       </c>
-      <c r="AB175" t="s">
+      <c r="AA175" t="s">
         <v>307</v>
+      </c>
+      <c r="AB175">
+        <v>31.202183381686979</v>
       </c>
     </row>
     <row r="176" spans="1:28" x14ac:dyDescent="0.25">
@@ -13059,8 +13581,11 @@
       <c r="S176">
         <v>0.49899999999999989</v>
       </c>
-      <c r="AB176" t="s">
+      <c r="AA176" t="s">
         <v>309</v>
+      </c>
+      <c r="AB176">
+        <v>37.476520402140792</v>
       </c>
     </row>
     <row r="177" spans="1:28" x14ac:dyDescent="0.25">
@@ -13118,8 +13643,11 @@
       <c r="S177">
         <v>0.50566666666666671</v>
       </c>
-      <c r="AB177" t="s">
+      <c r="AA177" t="s">
         <v>311</v>
+      </c>
+      <c r="AB177">
+        <v>45.900574842610688</v>
       </c>
     </row>
     <row r="178" spans="1:28" x14ac:dyDescent="0.25">
@@ -13177,8 +13705,11 @@
       <c r="S178">
         <v>0.45850000000000002</v>
       </c>
-      <c r="AB178" t="s">
+      <c r="AA178" t="s">
         <v>313</v>
+      </c>
+      <c r="AB178">
+        <v>47.401556521870852</v>
       </c>
     </row>
     <row r="179" spans="1:28" x14ac:dyDescent="0.25">
@@ -13236,8 +13767,11 @@
       <c r="S179">
         <v>0.504</v>
       </c>
-      <c r="AB179" t="s">
+      <c r="AA179" t="s">
         <v>315</v>
+      </c>
+      <c r="AB179">
+        <v>44.742071799271457</v>
       </c>
     </row>
     <row r="180" spans="1:28" x14ac:dyDescent="0.25">
@@ -13295,8 +13829,11 @@
       <c r="S180">
         <v>0.45466666666666661</v>
       </c>
-      <c r="AB180" t="s">
+      <c r="AA180" t="s">
         <v>317</v>
+      </c>
+      <c r="AB180">
+        <v>44.034322879772702</v>
       </c>
     </row>
     <row r="181" spans="1:28" x14ac:dyDescent="0.25">
@@ -13354,8 +13891,11 @@
       <c r="S181">
         <v>0.48849999999999999</v>
       </c>
-      <c r="AB181" t="s">
+      <c r="AA181" t="s">
         <v>319</v>
+      </c>
+      <c r="AB181">
+        <v>54.200728251785151</v>
       </c>
     </row>
     <row r="182" spans="1:28" x14ac:dyDescent="0.25">
@@ -13413,8 +13953,11 @@
       <c r="S182">
         <v>0.46899999999999997</v>
       </c>
-      <c r="AB182" t="s">
+      <c r="AA182" t="s">
         <v>321</v>
+      </c>
+      <c r="AB182">
+        <v>39.388003762164153</v>
       </c>
     </row>
     <row r="183" spans="1:28" x14ac:dyDescent="0.25">
@@ -13472,8 +14015,11 @@
       <c r="S183">
         <v>0.47883333333333339</v>
       </c>
-      <c r="AB183" t="s">
+      <c r="AA183" t="s">
         <v>323</v>
+      </c>
+      <c r="AB183">
+        <v>42.782906670636201</v>
       </c>
     </row>
     <row r="184" spans="1:28" x14ac:dyDescent="0.25">
@@ -13525,8 +14071,11 @@
       <c r="S184">
         <v>0.62883333333333324</v>
       </c>
-      <c r="AB184" t="s">
+      <c r="AA184" t="s">
         <v>325</v>
+      </c>
+      <c r="AB184">
+        <v>45.559191564172401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
loop para las variables, corregido SEQ5, ojo solo usar unique
</commit_message>
<xml_diff>
--- a/Numex_preliminar_base.xlsx
+++ b/Numex_preliminar_base.xlsx
@@ -1361,6 +1361,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AB184"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="18" max="18" width="22.85546875" customWidth="1"/>
+    <col min="19" max="19" width="15.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
@@ -6247,8 +6251,14 @@
       <c r="I64">
         <v>0.47866451539592519</v>
       </c>
+      <c r="J64">
+        <v>-33.6</v>
+      </c>
       <c r="K64">
         <v>1.4613558931996369E-2</v>
+      </c>
+      <c r="L64">
+        <v>1.37</v>
       </c>
       <c r="M64">
         <v>0.46982934570328277</v>

</xml_diff>